<commit_message>
Added queue version of Calculate Security Hash assignment
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\uipath\Calculate_Client_Security_Hash\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7145BA64-1C26-4D78-B973-8EE6CF722E77}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C67951D-471C-47C5-BA3E-A9FA0110C28F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="56">
   <si>
     <t>Name</t>
   </si>
@@ -156,9 +156,6 @@
     <t xml:space="preserve">The maximum number of consecutive system exceptions was reached. </t>
   </si>
   <si>
-    <t>ProcessABCQueue</t>
-  </si>
-  <si>
     <t>System1_URL</t>
   </si>
   <si>
@@ -190,6 +187,12 @@
   </si>
   <si>
     <t>https://acme-test.uipath.com/</t>
+  </si>
+  <si>
+    <t>items</t>
+  </si>
+  <si>
+    <t>Security_Hash</t>
   </si>
 </sst>
 </file>
@@ -615,7 +618,7 @@
         <v>23</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>21</v>
@@ -625,7 +628,9 @@
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="2"/>
+      <c r="B3" s="2" t="s">
+        <v>55</v>
+      </c>
       <c r="C3" s="4" t="s">
         <v>31</v>
       </c>
@@ -636,7 +641,7 @@
         <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>22</v>
@@ -645,44 +650,44 @@
     <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>48</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
       <c r="A11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>51</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>53</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>